<commit_message>
Remove building info extraction.
</commit_message>
<xml_diff>
--- a/templates/consolidated-data-template.xlsx
+++ b/templates/consolidated-data-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\super\Documents\arbaiza-consulting\environmental-sensor-poc\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6CCA266-C2C1-473B-8F8E-5FFA654168DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4217B9B1-D15B-41AA-B533-B489882749FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,8 +21,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">device_readings_daily!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">device_readings_last1000!$A$1:$K$1001</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">devices!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">sensors!$A$1:$K$398</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">devices!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">sensors!$A$1:$E$398</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
   <si>
     <t>Source</t>
   </si>
@@ -52,21 +52,6 @@
   </si>
   <si>
     <t>SensorTypes</t>
-  </si>
-  <si>
-    <t>DeviceSerialFromName</t>
-  </si>
-  <si>
-    <t>BuildingID</t>
-  </si>
-  <si>
-    <t>Building</t>
-  </si>
-  <si>
-    <t>Room</t>
-  </si>
-  <si>
-    <t>CardinalDirection</t>
   </si>
   <si>
     <t>SensorID</t>
@@ -449,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -457,14 +442,9 @@
     <col min="3" max="3" width="27.6640625" customWidth="1"/>
     <col min="4" max="5" width="50.77734375" customWidth="1"/>
     <col min="6" max="6" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -483,82 +463,44 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04DE2CC4-DFC8-4699-B107-22BCD5E3F531}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.109375" customWidth="1"/>
-    <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="43.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K398" xr:uid="{04DE2CC4-DFC8-4699-B107-22BCD5E3F531}"/>
+  <autoFilter ref="A1:E398" xr:uid="{04DE2CC4-DFC8-4699-B107-22BCD5E3F531}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -585,31 +527,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -646,7 +588,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -655,19 +597,19 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>